<commit_message>
chrome and main site
</commit_message>
<xml_diff>
--- a/ParabankAutomation/src/test/resources/TestData.xlsx
+++ b/ParabankAutomation/src/test/resources/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{4FFBC8E5-B9EF-4982-A146-ACC2DB4BF875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{ADDE251D-1578-4786-AF90-F11186E73497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DB95F208-3720-4456-9685-8E2D79731C20}"/>
   </bookViews>
@@ -12,7 +12,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:N6"/>
+  <oleSize ref="A1:P10"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -72,13 +72,13 @@
     <t>987-123</t>
   </si>
   <si>
-    <t>testnguser05</t>
-  </si>
-  <si>
-    <t>TestNG 05</t>
-  </si>
-  <si>
     <t>User 05</t>
+  </si>
+  <si>
+    <t>TestNG 06</t>
+  </si>
+  <si>
+    <t>testnguser06</t>
   </si>
 </sst>
 </file>
@@ -512,7 +512,7 @@
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>14</v>
@@ -533,7 +533,7 @@
         <v>15</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>12</v>
@@ -566,7 +566,7 @@
     </row>
     <row r="2" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Added Negative Login validation
</commit_message>
<xml_diff>
--- a/ParabankAutomation/src/test/resources/TestData.xlsx
+++ b/ParabankAutomation/src/test/resources/TestData.xlsx
@@ -3,16 +3,17 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{6CD92AF7-19AB-479C-83EB-E87A52B048E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{D4B3C6D9-3307-4BBA-B628-03B003526F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DB95F208-3720-4456-9685-8E2D79731C20}"/>
+    <workbookView xWindow="10752" yWindow="0" windowWidth="12324" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{DB95F208-3720-4456-9685-8E2D79731C20}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:L13"/>
+  <oleSize ref="A1:H17"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
   <si>
     <t>FirstName</t>
   </si>
@@ -79,6 +80,12 @@
   </si>
   <si>
     <t>testnguser04</t>
+  </si>
+  <si>
+    <t>invaliduser</t>
+  </si>
+  <si>
+    <t>invalidpass</t>
   </si>
 </sst>
 </file>
@@ -575,4 +582,34 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6295BCE6-402A-4372-84A5-FCA5379971BF}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>